<commit_message>
feat(i18n): adicionar suporte a idiomas inglês, espanhol e português feat(locale): implementar provider para gerenciamento de seleção de idioma
</commit_message>
<xml_diff>
--- a/Themas.xlsx
+++ b/Themas.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="41">
   <si>
     <t xml:space="preserve">Nome</t>
   </si>
@@ -52,18 +52,6 @@
     <t xml:space="preserve">On Error Container</t>
   </si>
   <si>
-    <t xml:space="preserve">Surface Dim</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Surface</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Surface Bright</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inverse Surface</t>
-  </si>
-  <si>
     <t xml:space="preserve">Relva</t>
   </si>
   <si>
@@ -94,15 +82,6 @@
     <t xml:space="preserve">#ffdad6</t>
   </si>
   <si>
-    <t xml:space="preserve">#d7dbd4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#f6fbf3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#2d322c</t>
-  </si>
-  <si>
     <t xml:space="preserve">Dark</t>
   </si>
   <si>
@@ -130,15 +109,6 @@
     <t xml:space="preserve">#93000a</t>
   </si>
   <si>
-    <t xml:space="preserve">#101510</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#353a35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#dfe4dc</t>
-  </si>
-  <si>
     <t xml:space="preserve">Outono</t>
   </si>
   <si>
@@ -157,15 +127,6 @@
     <t xml:space="preserve">#f5e1a7</t>
   </si>
   <si>
-    <t xml:space="preserve">#e8d6d2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#fff8f6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#392e2b</t>
-  </si>
-  <si>
     <t xml:space="preserve">#ffb5a0</t>
   </si>
   <si>
@@ -182,15 +143,6 @@
   </si>
   <si>
     <t xml:space="preserve">#534619</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#1a110f</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#423734</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#f1dfda</t>
   </si>
 </sst>
 </file>
@@ -200,7 +152,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -221,6 +173,11 @@
       <name val="Arial"/>
       <family val="0"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -240,9 +197,9 @@
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin"/>
-      <right/>
-      <top/>
-      <bottom/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
@@ -271,16 +228,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -407,224 +368,179 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
-  <sheetFormatPr defaultColWidth="17.6796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="17.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7.81"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="8.59"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="9.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="9.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="9.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="16.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="19.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="17.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="17.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16381" style="0" width="17.68"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="0" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="0" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="0" t="s">
+      <c r="B2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="0" t="s">
+      <c r="C2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="0" t="s">
+      <c r="D2" s="3" t="s">
         <v>13</v>
       </c>
+      <c r="E2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>19</v>
+      </c>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="0" t="s">
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="0" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" s="0" t="s">
-        <v>17</v>
-      </c>
-      <c r="E2" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="F2" s="0" t="s">
+      <c r="G4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G2" s="1" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="I2" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="J2" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="K2" s="0" t="s">
+      <c r="C5" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="L2" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="M2" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="N2" s="0" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="C3" s="0" t="s">
+      <c r="G5" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="J5" s="3" t="s">
         <v>28</v>
-      </c>
-      <c r="D3" s="0" t="s">
-        <v>29</v>
-      </c>
-      <c r="E3" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="F3" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="H3" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="I3" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="J3" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="K3" s="0" t="s">
-        <v>36</v>
-      </c>
-      <c r="L3" s="0" t="s">
-        <v>36</v>
-      </c>
-      <c r="M3" s="0" t="s">
-        <v>37</v>
-      </c>
-      <c r="N3" s="0" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>39</v>
-      </c>
-      <c r="B4" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="D4" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="E4" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="F4" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="H4" s="0" t="s">
-        <v>43</v>
-      </c>
-      <c r="I4" s="0" t="s">
-        <v>44</v>
-      </c>
-      <c r="J4" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="K4" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="L4" s="0" t="s">
-        <v>46</v>
-      </c>
-      <c r="M4" s="0" t="s">
-        <v>46</v>
-      </c>
-      <c r="N4" s="0" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="D5" s="0" t="s">
-        <v>49</v>
-      </c>
-      <c r="E5" s="0" t="s">
-        <v>50</v>
-      </c>
-      <c r="F5" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="H5" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="I5" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="J5" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="K5" s="0" t="s">
-        <v>54</v>
-      </c>
-      <c r="L5" s="0" t="s">
-        <v>54</v>
-      </c>
-      <c r="M5" s="0" t="s">
-        <v>55</v>
-      </c>
-      <c r="N5" s="0" t="s">
-        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>